<commit_message>
Add Celemony Melodyne and audit vocal chains
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/plugin_usage_semantic_hybrid_corrected.xlsx
+++ b/plugin_usage_semantic_hybrid_corrected.xlsx
@@ -1,37 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Навигация" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Бочка" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Snare Clap" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Томы Перкуссия" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Overheads" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Drum Room" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Drum Bus" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Бас-гитара" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 808 Synth Bass" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Lead Vocal" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Backing Vocals" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Речь Podcast" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Электрогитара" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Акустическая" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Piano Keys" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Synth Pads" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Strings Ensemble" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 FX Sound Design" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 Instrument Bus" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 Mix Bus" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 Mastering" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все цепочки" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Семейства плагинов" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Полный каталог" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Маршрутизация" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Навигация" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01 Бочка" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02 Snare Clap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03 Томы Перкуссия" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="04 Overheads" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05 Drum Room" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06 Drum Bus" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07 Бас-гитара" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="08 808 Synth Bass" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="09 Lead Vocal" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10 Backing Vocals" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11 Речь Podcast" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="12 Электрогитара" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="13 Акустическая" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="14 Piano Keys" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="15 Synth Pads" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="16 Strings Ensemble" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="17 FX Sound Design" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="18 Instrument Bus" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="19 Mix Bus" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="20 Mastering" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Все цепочки" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Семейства плагинов" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Полный каталог" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Маршрутизация" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -902,7 +902,7 @@
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="SemanticCatalog" displayName="SemanticCatalog" ref="A4:K368" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="SemanticCatalog" displayName="SemanticCatalog" ref="A4:K369" headerRowCount="1">
   <autoFilter ref="A4:K368"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Большая категория"/>
@@ -2196,7 +2196,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="27" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
@@ -2982,7 +2981,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="27" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
@@ -3735,7 +3733,6 @@
       </c>
       <c r="G7" s="11" t="inlineStr"/>
     </row>
-    <row r="8"/>
     <row r="9" ht="27" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -4264,7 +4261,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="27" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
@@ -5107,7 +5103,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="27" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -5794,7 +5789,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="27" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -6544,7 +6538,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="27" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
@@ -7275,7 +7268,6 @@
       </c>
       <c r="G6" s="11" t="inlineStr"/>
     </row>
-    <row r="7"/>
     <row r="8" ht="27" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
@@ -8023,7 +8015,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="27" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
@@ -8796,7 +8787,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="27" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
@@ -9599,7 +9589,6 @@
       </c>
       <c r="G11" s="11" t="inlineStr"/>
     </row>
-    <row r="12"/>
     <row r="13" ht="27" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
@@ -10483,7 +10472,6 @@
       </c>
       <c r="G10" s="11" t="inlineStr"/>
     </row>
-    <row r="11"/>
     <row r="12" ht="27" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
@@ -11262,7 +11250,6 @@
       </c>
       <c r="G10" s="11" t="inlineStr"/>
     </row>
-    <row r="11"/>
     <row r="12" ht="27" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
@@ -14440,37 +14427,38 @@
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>★ Waves Tune
+          <t>★ Celemony Melodyne
+★ Waves Tune
 ★ Waves Tune Real-Time</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Waves Tune, Waves Tune Real-Time</t>
+          <t>Celemony Melodyne, Waves Tune, Waves Tune Real-Time</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>Исправление высоты и timing/pitch отдельных нот.</t>
+          <t>Исправление высоты, timing и длины отдельных нот.</t>
         </is>
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>Graphical — прозрачно и вручную; real-time — быстро или как эффект.</t>
+          <t>Melodyne и Waves Tune — детальная graphical correction; Tune Real-Time — быстрый automatic/creative режим.</t>
         </is>
       </c>
       <c r="G14" s="19" t="inlineStr">
         <is>
-          <t>Lead vocal, monophonic instruments.</t>
+          <t>Lead vocal, backing vocals, monophonic instruments.</t>
         </is>
       </c>
       <c r="H14" s="19" t="inlineStr">
         <is>
-          <t>После editing, до основной dynamics.</t>
+          <t>После comping/editing, до EQ, compression и time effects.</t>
         </is>
       </c>
       <c r="I14" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="76" customHeight="1">
@@ -17272,7 +17260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K368"/>
+  <dimension ref="A1:K369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -36855,7 +36843,63 @@
       </c>
       <c r="K368" s="52" t="inlineStr"/>
     </row>
-    <row r="369" ht="64" customHeight="1"/>
+    <row r="369" ht="64" customHeight="1">
+      <c r="A369" s="86" t="inlineStr">
+        <is>
+          <t>Cleanup и restoration</t>
+        </is>
+      </c>
+      <c r="B369" s="52" t="inlineStr">
+        <is>
+          <t>Pitch correction</t>
+        </is>
+      </c>
+      <c r="C369" s="53" t="inlineStr">
+        <is>
+          <t>Celemony Melodyne</t>
+        </is>
+      </c>
+      <c r="D369" s="52" t="inlineStr">
+        <is>
+          <t>Celemony</t>
+        </is>
+      </c>
+      <c r="E369" s="52" t="inlineStr">
+        <is>
+          <t>Graphical note-based pitch and timing editor</t>
+        </is>
+      </c>
+      <c r="F369" s="52" t="inlineStr">
+        <is>
+          <t>Lead vocal, backing vocals, monophonic instruments</t>
+        </is>
+      </c>
+      <c r="G369" s="52" t="inlineStr">
+        <is>
+          <t>Показывает ноты как blobs и позволяет вручную исправлять pitch, timing и длину; набор дополнительных tools зависит от edition</t>
+        </is>
+      </c>
+      <c r="H369" s="52" t="inlineStr">
+        <is>
+          <t>Waves Tune, Waves Tune Real-Time</t>
+        </is>
+      </c>
+      <c r="I369" s="52" t="inlineStr">
+        <is>
+          <t>Основной</t>
+        </is>
+      </c>
+      <c r="J369" s="52" t="inlineStr">
+        <is>
+          <t>Сначала comping и clip editing. Использовать через ARA или первым insert на чистом dry-сигнале; исправлять только слышимые ошибки. Возможности Essential, Assistant, Editor и Studio различаются.</t>
+        </is>
+      </c>
+      <c r="K369" s="4" t="inlineStr">
+        <is>
+          <t>https://www.celemony.com/en/melodyne/what-is-melodyne</t>
+        </is>
+      </c>
+    </row>
     <row r="370" ht="64" customHeight="1"/>
     <row r="371" ht="64" customHeight="1"/>
     <row r="372" ht="64" customHeight="1"/>
@@ -36924,6 +36968,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K354" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K362" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K365" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K369" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -36936,7 +36981,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId52"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId53"/>
   </tableParts>
 </worksheet>
 </file>
@@ -37352,7 +37397,6 @@
       </c>
       <c r="G9" s="11" t="inlineStr"/>
     </row>
-    <row r="10"/>
     <row r="11" ht="27" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
@@ -38155,7 +38199,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="27" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
@@ -38872,7 +38915,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="27" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -39595,7 +39637,6 @@
       </c>
       <c r="G11" s="11" t="inlineStr"/>
     </row>
-    <row r="12"/>
     <row r="13" ht="27" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
@@ -40553,7 +40594,6 @@
       </c>
       <c r="G11" s="11" t="inlineStr"/>
     </row>
-    <row r="12"/>
     <row r="13" ht="27" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
@@ -41480,7 +41520,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="27" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
@@ -42343,7 +42382,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="27" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>

</xml_diff>